<commit_message>
Added DDT Test Cases
</commit_message>
<xml_diff>
--- a/TestData/Faker_Data.xlsx
+++ b/TestData/Faker_Data.xlsx
@@ -390,13 +390,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="25.6640625" customWidth="1" min="2" max="2"/>
     <col width="30.21875" customWidth="1" min="3" max="3"/>
     <col width="29.6640625" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21.5546875" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,6 +432,16 @@
           <t>Status message</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Expected_message</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Test cases status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -437,7 +449,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>waglenilima</t>
+          <t>tanveernagi</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -447,17 +459,27 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>surabarkha@example.com</t>
+          <t>kandariya@example.org</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>+916371640050</t>
+          <t>7409698672</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -467,7 +489,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>dbail</t>
+          <t>mahajanekalinga</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -477,17 +499,27 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>mannranveer@example.org</t>
+          <t>omnikita@example.org</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>02509565628</t>
+          <t>+918730180055</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -497,7 +529,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>yashasvishenoy</t>
+          <t>kwali</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -507,17 +539,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pallaeta@example.org</t>
+          <t>mohini20@example.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+917677181566</t>
+          <t>+917738817290</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -527,7 +569,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>nitesh14</t>
+          <t>morevamakshi</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -537,17 +579,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>urishilla76@example.net</t>
+          <t>yratti@example.com</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>00078535750</t>
+          <t>00079383602</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -557,7 +609,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>geraryan</t>
+          <t>usaran</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -567,12 +619,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>chakradharkurian@example.com</t>
+          <t>jonathangarde@example.org</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6969718021</t>
+          <t>6000747512</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -580,154 +632,14 @@
           <t>User created successfully</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>menonqushi</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>QaTest#2026</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>xkeer@example.com</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>00030495396</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>User created successfully</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>tanveer19</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>QaTest#2026</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>mpatla@example.net</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>03797336250</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>User created successfully</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>duabalhaar</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>QaTest#2026</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>zaidpurohit@example.org</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>9259081927</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>User created successfully</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>jhalak30</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>QaTest#2026</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>qarin76@example.com</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>04102100718</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>User created successfully</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>wagleishaan</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>QaTest#2026</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>lilareddy@example.org</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>+914297324937</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>User created successfully</t>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>User created successfully</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Customer management Test Cases adding
</commit_message>
<xml_diff>
--- a/TestData/Faker_Data.xlsx
+++ b/TestData/Faker_Data.xlsx
@@ -449,7 +449,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>tanveernagi</t>
+          <t>pallavi28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -459,12 +459,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>kandariya@example.org</t>
+          <t>benjaminpau@example.net</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7409698672</t>
+          <t>02780625828</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>mahajanekalinga</t>
+          <t>ldalal</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -499,12 +499,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>omnikita@example.org</t>
+          <t>zayansangha@example.org</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+918730180055</t>
+          <t>4090448874</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -529,7 +529,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>kwali</t>
+          <t>wadhwabhavika</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -539,12 +539,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>mohini20@example.com</t>
+          <t>hmammen@example.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+917738817290</t>
+          <t>7939885517</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>morevamakshi</t>
+          <t>onkarkade</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>yratti@example.com</t>
+          <t>uaurora@example.com</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>00079383602</t>
+          <t>03683492844</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>usaran</t>
+          <t>twadhwa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -619,12 +619,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>jonathangarde@example.org</t>
+          <t>msridhar@example.net</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6000747512</t>
+          <t>0267574985</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>